<commit_message>
Ajouts articles veille, mise à jour excel, modif projets
</commit_message>
<xml_diff>
--- a/docs/veille.xlsx
+++ b/docs/veille.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="104">
   <si>
     <t>Date</t>
   </si>
@@ -31,6 +31,12 @@
   </si>
   <si>
     <t>Ubisoft investit en R&amp;D sur des outils permettant aux joueurs de pouvoir avoir des conversations "naturelles" avec des personnages non-joueurs dans les jeux vidéos.</t>
+  </si>
+  <si>
+    <t>L'IA facilite le travail des artistes/deisgners ?</t>
+  </si>
+  <si>
+    <t>Article expliquant l'utilisation de l'IA comme un outil d'aide à la création de terrains, de détails dans de grands univers pour les artistes, plutôt que comme un remplacement.</t>
   </si>
   <si>
     <t>EA utilise l'IA pour presque tout, effet néfaste</t>
@@ -98,15 +104,242 @@
   <si>
     <t>Le CEO de Larian (studio qui a créé Baldur's Gate 3) indique qu'ils utilisent bien l'IA mais pour "explorer des choses" et non pas remplacer les artistes.</t>
   </si>
+  <si>
+    <t>Décision radicale face à accusation d'IA</t>
+  </si>
+  <si>
+    <t>Face aux accusations d'utilisation d'IA, le studio Urban Games décide de repartir sur feuille blanche et d'adopter une direction artistique différente pour empêcher tout soupçon.</t>
+  </si>
+  <si>
+    <t>Craintes quant à nouvelle responsable XBox</t>
+  </si>
+  <si>
+    <t>La nouvelle responsable de la division de jeu chez Microsoft est ancienne présidente de CoreAI ; cependant, elle affirme ne pas vouloir faire de jeux "sans âme".</t>
+  </si>
+  <si>
+    <t>IA Générative dans les jeux-vidéos</t>
+  </si>
+  <si>
+    <t>Article récapitulant les différentes utilisations de l'IA générative dans les jeux avec des exemples concrets, noms d'outils (Nvidia ACE, Ubisoft NEO...), statistiques...</t>
+  </si>
+  <si>
+    <t>L'IA Révolutionne le game design</t>
+  </si>
+  <si>
+    <t>Autres exemples d'IA générative pour le game design avec beaucoup d'outils (Roblox Cube 3D, Ubisoft Ghostwriter, GameDriver, Test.AI), stats, perspectives d'avenir...</t>
+  </si>
+  <si>
+    <t>Réflexion quant à la nature de la révolution</t>
+  </si>
+  <si>
+    <t>L'intelligence Artificielle a du mal à comprendre l'humain et le côté artistique va donc sûrement plus évoluer vers l'écriture des personnages, ou des styles imparfaits, particuliers.</t>
+  </si>
+  <si>
+    <t>L'IA n'aide pas les artistes, au contraire</t>
+  </si>
+  <si>
+    <t>Dans l'industrie du jeu vidéo, l'IA freine l'imagination des artistes avec tous les clients générant des concept art très détaillés, ne laissant pas place à l'imagination</t>
+  </si>
+  <si>
+    <t>10 prédictions sur l'utilisation de l'IA dans jeu</t>
+  </si>
+  <si>
+    <t>10 prédictions concernant l'augmentation de l'utilisation de l'IA, les conséquences (pénuries) et les réactions pour l'année 2026</t>
+  </si>
+  <si>
+    <t>Nouvel assistant IA qui jouera pour nous</t>
+  </si>
+  <si>
+    <t>Microsoft ont annoncé un futur outil d'IA qui pourra jouer à notre place afin de débloquer le joueur dans des cas ou le niveau / combat est trop difficile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blizzard contre la génération par IA </t>
+  </si>
+  <si>
+    <t>Leo Kaliski, compositeur principal de World of Warcraft: Midnight, se dit très chanceux et heureux de ne pas utiliser l'IA pour les musiques des jeux Blizzard (+ contrexemple voix)</t>
+  </si>
+  <si>
+    <t>La fin de Xbox au profit de l’IA</t>
+  </si>
+  <si>
+    <t>Seamus Blackley, l'un des créateurs de XBox, affirme que nous allons assister à la fin de XBox avec l'arrivée de Asha Sharma à la tête de XBox Gaming</t>
+  </si>
+  <si>
+    <t>"Nouvelle réalité" dans le game design</t>
+  </si>
+  <si>
+    <t>Questions éthiques sur l'IA, 84% des développeurs de jeux inquiétés par l'éthique quant à l'utilisation responsable de l'IA générative (GameNGen, DeepMind Genie, Unity Muse...)</t>
+  </si>
+  <si>
+    <t>Panorama utilisation IA dans jeux-vidéos</t>
+  </si>
+  <si>
+    <t>Panorama de l'utilisation de l'IA dans le domaine du jeu vidéo, quels studios intègrent IA, comment, quels sont les problèmes ... le tout avec des statistiques.</t>
+  </si>
+  <si>
+    <t>Différentes positions quant à l'IA dans le JV</t>
+  </si>
+  <si>
+    <t>Article parlant des différents points de vue sur l'IA et plus précisément sur la création de jeux-vidéos (passant par les "AIGeeks", les "FuckAI" et même l'entre-deux.</t>
+  </si>
+  <si>
+    <t>IA et Gaming : la révolution Muse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'article explore l'évolution de l'IA dans le gaming, focalisé sur Muse de Microsoft, un modèle génératif entraîné sur Bleeding Edge pour prototypage rapide et préservation de jeux, malgré critiques sur l'emploi et la créativité. </t>
+  </si>
+  <si>
+    <t>AI Slop Infects Game Promotion and Reviews</t>
+  </si>
+  <si>
+    <t>Article qui explique comment des contenus générés par IA (« AI slop ») envahissent la promo et les critiques de jeux vidéo, avec les cas TikTok/Usual June et la review IA de VideoGamer retirée par Metacritic.</t>
+  </si>
+  <si>
+    <t>Après Sony, chez Xbox aussi on veut que l'IA finisse vos jeux à votre place</t>
+  </si>
+  <si>
+    <t>Article sur un brevet Xbox décrivant une IA capable de finir les jeux à la place du joueur quand il est bloqué, et sur les risques d’un « gaming zéro effort » qui vide l’expérience de son intérêt.</t>
+  </si>
+  <si>
+    <t>Aura 12.0 Beta</t>
+  </si>
+  <si>
+    <t>Aura 12.0 beta, la nouvelle version de l’assistant IA multi‑agents de Ramen pour Unreal Engine, qui améliore fortement l’édition de Blueprints, l’animation/rigging et l’automatisation du workflow de développement de jeux.</t>
+  </si>
+  <si>
+    <t>Unity Promises Deluge Of New Games Prompted Into Existence By AI</t>
+  </si>
+  <si>
+    <t>Nouvelle version de son outil Unity AI capable de générer des jeux « casual » jouables à partir de simples prompts en langage naturel, ce qui pourrait inonder le marché de jeux générés par IA de qualité discutable</t>
+  </si>
+  <si>
+    <t>Investissement dans l'IA par Koei Tecmo</t>
+  </si>
+  <si>
+    <t>Le studio de jeu Koei Tecmo a annoncé collaborer avec SpiralAI qui entrainent depuis des années leur modèle gepeto2 qui aura pour but de se mettre dans la peau des personnages pour leur donner vie</t>
+  </si>
+  <si>
+    <t>IA dans le développement de jeux, exemples d'applications</t>
+  </si>
+  <si>
+    <t>Article récapitulant les utilisations de l'IA générative par les studios de jeux, les bonnes pratiques, les problèmes et qui parle notamment de "AI powered game engine" et de personnalisation</t>
+  </si>
+  <si>
+    <t>IA bénéfique pour les artistes car utilisateur cherche authenticité</t>
+  </si>
+  <si>
+    <t>Troy Baker, musicien, acteur, et interprète de personnages de jeux-vidéos, annonce qu'il pense que les utilisateurs vont s'orienter vers les jeux-vidéos faits sans IA en réponse à l'émergence de l'IA</t>
+  </si>
+  <si>
+    <t>Statistiques sur l'avis des gamers sur la gen-AI dans les jeux-vidéos</t>
+  </si>
+  <si>
+    <t>Données issues d'un sondage envers des gamers qui montre les pourcentages de positivité / négativité envers la gen-AI, pour différencier selon âge, genre, et également l'utilisation de la gen-AI (artistique vs procédural)</t>
+  </si>
+  <si>
+    <t>xAI, studio de jeux-vidéos IA annoncé par Elon Musk</t>
+  </si>
+  <si>
+    <t>xAI est un studio de jeux-vidéos fondé par Elon Musk, qui affirme que l'on aura un "bon jeu vidéo jouable avant la fin de 2026, entièrement fait par IA"</t>
+  </si>
+  <si>
+    <t>IA révolutionne game design, catalyseur de créativité ?</t>
+  </si>
+  <si>
+    <t>Panorama des possibles utilisations de l'IA dans le game design avec témoignage d'Emma Rodriguez, qui affirme que la gen-IA ne remplace pas les artistes mais permet en réaliter de booster leur créativité</t>
+  </si>
+  <si>
+    <t>l’IA générative devient un repoussoir dans le jeu vidéo</t>
+  </si>
+  <si>
+    <t>Analyse du rejet croissant de l'IA générative par les développeurs lors de la GDC 2026</t>
+  </si>
+  <si>
+    <t>NVIDIA's Autonomous AI Characters Are Coming to Popular Games</t>
+  </si>
+  <si>
+    <t>NVIDIA annonce l'arrivée de personnages autonomes ACE capables de planifier des actions dans PUBG.</t>
+  </si>
+  <si>
+    <t>L’IA dans les jeux vidéo : Des positions qui s’éloignent</t>
+  </si>
+  <si>
+    <t>Enquête sur les tensions sociales et les licenciements liés à l'adoption massive de l'IA dans les studios.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elon Musk: un jeu vidéo généré par IA prévu avant fin 2026
+</t>
+  </si>
+  <si>
+    <t>Elon Musk annonce son ambition de produire un jeu vidéo entièrement généré par IA d'ici fin 2026.</t>
+  </si>
+  <si>
+    <t>2025-17-09</t>
+  </si>
+  <si>
+    <t>How Generative-AI Is Changing Gaming in 2025 (And What That Means for You)</t>
+  </si>
+  <si>
+    <t>Étude sur l'impact de l'IA générative sur le level design et le comportement des PNJ dans les jeux AAA.</t>
+  </si>
+  <si>
+    <t>Jeux vidéo et AI Act : la partie ne fait que commencer</t>
+  </si>
+  <si>
+    <t>Analyse juridique de l'impact de l'AI Act européen sur les studios de développement de jeux vidéo.</t>
+  </si>
+  <si>
+    <t>Jeu vidéo en 2025: notre grand récap des 10 tendances majeures de l’année</t>
+  </si>
+  <si>
+    <t>Bilan des 10 tendances majeures de 2025, où l'IA s'impose comme outil de survie économique.</t>
+  </si>
+  <si>
+    <t>The Impact Of AI on Video Game Development in 2025</t>
+  </si>
+  <si>
+    <t>Comment l'IA améliore l'assurance qualité (QA) et le débogage en simulant des milliers de tests.</t>
+  </si>
+  <si>
+    <t>Tencent Games unveils AI tools</t>
+  </si>
+  <si>
+    <t>Tencent dévoile VISVISE, une suite d'IA capable de générer des animations 3D et de gérer automatiquement le rigging des personnages.</t>
+  </si>
+  <si>
+    <t>Racing Lab : Quand l’IA devient votre coach de pilotage</t>
+  </si>
+  <si>
+    <t>Moza Racing dévoile à la GDC 2026 une IA de "Reinforcement Learning" qui analyse le pilotage du joueur pour corriger sa trajectoire et sa mémoire musculaire en temps réel.</t>
+  </si>
+  <si>
+    <t>2026 : les tendances du jeu vidéo vues par Nintendo, Sony, Microsoft</t>
+  </si>
+  <si>
+    <t>Analyse des tendances 2026 : l'IA permet désormais des rencontres scriptées et adaptatives dans les mondes ouverts, renforçant l'immersion narrative.</t>
+  </si>
+  <si>
+    <t>NVIDIA GeForce ON à la GDC 2026 : focus RTX, IA et path tracing, pas de nouveau GPU</t>
+  </si>
+  <si>
+    <t>NVIDIA profite de la GDC 2026 pour montrer comment l'IA et le "path tracing" permettent désormais un rendu photoréaliste en temps réel sans sacrifier les FPS.</t>
+  </si>
+  <si>
+    <t>Les studios AAA virent leurs développeurs au nom de l'IA et s'en vantent.</t>
+  </si>
+  <si>
+    <t>Enquête sur le paradoxe de 2026 : alors que les studios AAA licencient au nom de l'IA, les développeurs solos s'en servent massivement pour concurrencer les blockbusters.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -138,6 +371,12 @@
     <font>
       <u/>
       <sz val="11.0"/>
+      <color rgb="FF467886"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11.0"/>
       <color theme="10"/>
       <name val="Aptos Narrow"/>
     </font>
@@ -154,10 +393,13 @@
       <name val="Arial"/>
     </font>
     <font>
-      <u/>
-      <sz val="11.0"/>
-      <color rgb="FF467886"/>
+      <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -186,7 +428,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="21">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -202,16 +444,22 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="center"/>
+    </xf>
     <xf borderId="1" fillId="2" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -220,20 +468,29 @@
     <xf borderId="0" fillId="2" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="center"/>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -449,8 +706,8 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="17.5"/>
-    <col customWidth="1" min="2" max="2" width="38.0"/>
-    <col customWidth="1" min="3" max="3" width="149.25"/>
+    <col customWidth="1" min="2" max="2" width="74.5"/>
+    <col customWidth="1" min="3" max="3" width="183.13"/>
     <col customWidth="1" min="4" max="6" width="11.5"/>
     <col customWidth="1" min="7" max="26" width="10.63"/>
   </cols>
@@ -524,9 +781,15 @@
       <c r="Z2" s="2"/>
     </row>
     <row r="3" ht="39.75" customHeight="1">
-      <c r="A3" s="1"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
+      <c r="A3" s="3">
+        <v>45245.0</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>6</v>
+      </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
@@ -552,14 +815,14 @@
       <c r="Z3" s="2"/>
     </row>
     <row r="4" ht="39.75" customHeight="1">
-      <c r="A4" s="5">
+      <c r="A4" s="7">
         <v>45959.0</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>5</v>
+      <c r="B4" s="8" t="s">
+        <v>7</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>6</v>
+      <c r="C4" s="9" t="s">
+        <v>8</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
@@ -590,10 +853,10 @@
         <v>45961.0</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
@@ -620,14 +883,14 @@
       <c r="Z5" s="2"/>
     </row>
     <row r="6" ht="39.75" customHeight="1">
-      <c r="A6" s="5">
+      <c r="A6" s="7">
         <v>45962.0</v>
       </c>
-      <c r="B6" s="8" t="s">
-        <v>9</v>
+      <c r="B6" s="10" t="s">
+        <v>11</v>
       </c>
-      <c r="C6" s="9" t="s">
-        <v>10</v>
+      <c r="C6" s="11" t="s">
+        <v>12</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -658,10 +921,10 @@
         <v>45962.0</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
@@ -688,14 +951,14 @@
       <c r="Z7" s="2"/>
     </row>
     <row r="8" ht="39.75" customHeight="1">
-      <c r="A8" s="10">
+      <c r="A8" s="12">
         <v>45964.0</v>
       </c>
-      <c r="B8" s="11" t="s">
-        <v>13</v>
+      <c r="B8" s="13" t="s">
+        <v>15</v>
       </c>
-      <c r="C8" s="12" t="s">
-        <v>14</v>
+      <c r="C8" s="14" t="s">
+        <v>16</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
@@ -725,11 +988,11 @@
       <c r="A9" s="3">
         <v>45964.0</v>
       </c>
-      <c r="B9" s="13" t="s">
-        <v>15</v>
+      <c r="B9" s="15" t="s">
+        <v>17</v>
       </c>
-      <c r="C9" s="14" t="s">
-        <v>16</v>
+      <c r="C9" s="6" t="s">
+        <v>18</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
@@ -759,11 +1022,11 @@
       <c r="A10" s="3">
         <v>45964.0</v>
       </c>
-      <c r="B10" s="13" t="s">
-        <v>17</v>
+      <c r="B10" s="15" t="s">
+        <v>19</v>
       </c>
-      <c r="C10" s="14" t="s">
-        <v>18</v>
+      <c r="C10" s="6" t="s">
+        <v>20</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
@@ -793,11 +1056,11 @@
       <c r="A11" s="3">
         <v>45964.0</v>
       </c>
-      <c r="B11" s="13" t="s">
-        <v>19</v>
+      <c r="B11" s="15" t="s">
+        <v>21</v>
       </c>
-      <c r="C11" s="14" t="s">
-        <v>20</v>
+      <c r="C11" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
@@ -827,11 +1090,11 @@
       <c r="A12" s="3">
         <v>45960.0</v>
       </c>
-      <c r="B12" s="13" t="s">
-        <v>21</v>
+      <c r="B12" s="15" t="s">
+        <v>23</v>
       </c>
-      <c r="C12" s="14" t="s">
-        <v>22</v>
+      <c r="C12" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -861,11 +1124,11 @@
       <c r="A13" s="3">
         <v>45965.0</v>
       </c>
-      <c r="B13" s="15" t="s">
-        <v>23</v>
+      <c r="B13" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="C13" s="14" t="s">
-        <v>24</v>
+      <c r="C13" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -895,11 +1158,11 @@
       <c r="A14" s="3">
         <v>46008.0</v>
       </c>
-      <c r="B14" s="13" t="s">
-        <v>25</v>
+      <c r="B14" s="15" t="s">
+        <v>27</v>
       </c>
-      <c r="C14" s="14" t="s">
-        <v>26</v>
+      <c r="C14" s="6" t="s">
+        <v>28</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
@@ -926,9 +1189,15 @@
       <c r="Z14" s="2"/>
     </row>
     <row r="15" ht="39.75" customHeight="1">
-      <c r="A15" s="1"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
+      <c r="A15" s="3">
+        <v>46076.0</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
@@ -954,9 +1223,15 @@
       <c r="Z15" s="2"/>
     </row>
     <row r="16" ht="39.75" customHeight="1">
-      <c r="A16" s="1"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
+      <c r="A16" s="3">
+        <v>46076.0</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>32</v>
+      </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
@@ -982,9 +1257,15 @@
       <c r="Z16" s="2"/>
     </row>
     <row r="17" ht="39.75" customHeight="1">
-      <c r="A17" s="1"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
+      <c r="A17" s="12">
+        <v>46076.0</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>34</v>
+      </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
@@ -1010,9 +1291,15 @@
       <c r="Z17" s="2"/>
     </row>
     <row r="18" ht="39.75" customHeight="1">
-      <c r="A18" s="1"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
+      <c r="A18" s="12">
+        <v>46069.0</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>36</v>
+      </c>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
@@ -1038,9 +1325,15 @@
       <c r="Z18" s="2"/>
     </row>
     <row r="19" ht="39.75" customHeight="1">
-      <c r="A19" s="1"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
+      <c r="A19" s="3">
+        <v>46081.0</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>38</v>
+      </c>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
@@ -1066,9 +1359,15 @@
       <c r="Z19" s="2"/>
     </row>
     <row r="20" ht="39.75" customHeight="1">
-      <c r="A20" s="1"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
+      <c r="A20" s="3">
+        <v>46030.0</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>40</v>
+      </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
@@ -1094,9 +1393,15 @@
       <c r="Z20" s="2"/>
     </row>
     <row r="21" ht="39.75" customHeight="1">
-      <c r="A21" s="1"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
+      <c r="A21" s="3">
+        <v>46036.0</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>42</v>
+      </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
@@ -1122,9 +1427,15 @@
       <c r="Z21" s="2"/>
     </row>
     <row r="22" ht="39.75" customHeight="1">
-      <c r="A22" s="1"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
+      <c r="A22" s="16">
+        <v>46085.0</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>44</v>
+      </c>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
@@ -1150,9 +1461,15 @@
       <c r="Z22" s="2"/>
     </row>
     <row r="23" ht="39.75" customHeight="1">
-      <c r="A23" s="1"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
+      <c r="A23" s="3">
+        <v>46083.0</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>46</v>
+      </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
@@ -1178,9 +1495,15 @@
       <c r="Z23" s="2"/>
     </row>
     <row r="24" ht="39.75" customHeight="1">
-      <c r="A24" s="1"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
+      <c r="A24" s="3">
+        <v>46084.0</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>48</v>
+      </c>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
@@ -1206,9 +1529,15 @@
       <c r="Z24" s="2"/>
     </row>
     <row r="25" ht="39.75" customHeight="1">
-      <c r="A25" s="1"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
+      <c r="A25" s="3">
+        <v>45579.0</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>50</v>
+      </c>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
@@ -1234,9 +1563,15 @@
       <c r="Z25" s="2"/>
     </row>
     <row r="26" ht="39.75" customHeight="1">
-      <c r="A26" s="1"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
+      <c r="A26" s="3">
+        <v>45251.0</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>52</v>
+      </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
@@ -1262,9 +1597,15 @@
       <c r="Z26" s="2"/>
     </row>
     <row r="27" ht="39.75" customHeight="1">
-      <c r="A27" s="1"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
+      <c r="A27" s="3">
+        <v>45978.0</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>54</v>
+      </c>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
       <c r="F27" s="2"/>
@@ -1290,9 +1631,15 @@
       <c r="Z27" s="2"/>
     </row>
     <row r="28" ht="39.75" customHeight="1">
-      <c r="A28" s="1"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
+      <c r="A28" s="3">
+        <v>45720.0</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>56</v>
+      </c>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
@@ -1318,11 +1665,17 @@
       <c r="Z28" s="2"/>
     </row>
     <row r="29" ht="39.75" customHeight="1">
-      <c r="A29" s="1"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
+      <c r="A29" s="3">
+        <v>46085.0</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D29" s="17"/>
+      <c r="E29" s="6"/>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
@@ -1346,9 +1699,15 @@
       <c r="Z29" s="2"/>
     </row>
     <row r="30" ht="39.75" customHeight="1">
-      <c r="A30" s="1"/>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
+      <c r="A30" s="3">
+        <v>46086.0</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
@@ -1374,9 +1733,15 @@
       <c r="Z30" s="2"/>
     </row>
     <row r="31" ht="39.75" customHeight="1">
-      <c r="A31" s="1"/>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
+      <c r="A31" s="12">
+        <v>46056.0</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>62</v>
+      </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
       <c r="F31" s="2"/>
@@ -1402,9 +1767,15 @@
       <c r="Z31" s="2"/>
     </row>
     <row r="32" ht="39.75" customHeight="1">
-      <c r="A32" s="1"/>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
+      <c r="A32" s="3">
+        <v>46070.0</v>
+      </c>
+      <c r="B32" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>64</v>
+      </c>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
@@ -1430,9 +1801,15 @@
       <c r="Z32" s="2"/>
     </row>
     <row r="33" ht="39.75" customHeight="1">
-      <c r="A33" s="1"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
+      <c r="A33" s="3">
+        <v>46089.0</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>66</v>
+      </c>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
       <c r="F33" s="2"/>
@@ -1458,9 +1835,15 @@
       <c r="Z33" s="2"/>
     </row>
     <row r="34" ht="39.75" customHeight="1">
-      <c r="A34" s="1"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
+      <c r="A34" s="3">
+        <v>45982.0</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>68</v>
+      </c>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
       <c r="F34" s="2"/>
@@ -1486,9 +1869,15 @@
       <c r="Z34" s="2"/>
     </row>
     <row r="35" ht="39.75" customHeight="1">
-      <c r="A35" s="1"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
+      <c r="A35" s="12">
+        <v>46028.0</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="C35" s="14" t="s">
+        <v>70</v>
+      </c>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
       <c r="F35" s="2"/>
@@ -1514,9 +1903,15 @@
       <c r="Z35" s="2"/>
     </row>
     <row r="36" ht="39.75" customHeight="1">
-      <c r="A36" s="1"/>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
+      <c r="A36" s="12">
+        <v>46009.0</v>
+      </c>
+      <c r="B36" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C36" s="14" t="s">
+        <v>72</v>
+      </c>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
       <c r="F36" s="2"/>
@@ -1542,9 +1937,15 @@
       <c r="Z36" s="2"/>
     </row>
     <row r="37" ht="39.75" customHeight="1">
-      <c r="A37" s="1"/>
-      <c r="B37" s="2"/>
-      <c r="C37" s="2"/>
+      <c r="A37" s="3">
+        <v>45947.0</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>74</v>
+      </c>
       <c r="D37" s="2"/>
       <c r="E37" s="2"/>
       <c r="F37" s="2"/>
@@ -1570,9 +1971,15 @@
       <c r="Z37" s="2"/>
     </row>
     <row r="38" ht="39.75" customHeight="1">
-      <c r="A38" s="1"/>
-      <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
+      <c r="A38" s="3">
+        <v>45666.0</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>76</v>
+      </c>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
       <c r="F38" s="2"/>
@@ -1598,9 +2005,15 @@
       <c r="Z38" s="2"/>
     </row>
     <row r="39" ht="39.75" customHeight="1">
-      <c r="A39" s="1"/>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
+      <c r="A39" s="3">
+        <v>46053.0</v>
+      </c>
+      <c r="B39" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>78</v>
+      </c>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
       <c r="F39" s="2"/>
@@ -1626,9 +2039,15 @@
       <c r="Z39" s="2"/>
     </row>
     <row r="40" ht="39.75" customHeight="1">
-      <c r="A40" s="1"/>
-      <c r="B40" s="2"/>
-      <c r="C40" s="2"/>
+      <c r="A40" s="3">
+        <v>45665.0</v>
+      </c>
+      <c r="B40" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>80</v>
+      </c>
       <c r="D40" s="2"/>
       <c r="E40" s="2"/>
       <c r="F40" s="2"/>
@@ -1654,9 +2073,15 @@
       <c r="Z40" s="2"/>
     </row>
     <row r="41" ht="39.75" customHeight="1">
-      <c r="A41" s="1"/>
-      <c r="B41" s="2"/>
-      <c r="C41" s="2"/>
+      <c r="A41" s="3">
+        <v>45978.0</v>
+      </c>
+      <c r="B41" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C41" s="18" t="s">
+        <v>82</v>
+      </c>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
       <c r="F41" s="2"/>
@@ -1682,9 +2107,15 @@
       <c r="Z41" s="2"/>
     </row>
     <row r="42" ht="39.75" customHeight="1">
-      <c r="A42" s="1"/>
-      <c r="B42" s="2"/>
-      <c r="C42" s="2"/>
+      <c r="A42" s="3">
+        <v>45938.0</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C42" s="19" t="s">
+        <v>84</v>
+      </c>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
       <c r="F42" s="2"/>
@@ -1710,9 +2141,15 @@
       <c r="Z42" s="2"/>
     </row>
     <row r="43" ht="39.75" customHeight="1">
-      <c r="A43" s="1"/>
-      <c r="B43" s="2"/>
-      <c r="C43" s="2"/>
+      <c r="A43" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="B43" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="C43" s="19" t="s">
+        <v>87</v>
+      </c>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
       <c r="F43" s="2"/>
@@ -1738,9 +2175,15 @@
       <c r="Z43" s="2"/>
     </row>
     <row r="44" ht="39.75" customHeight="1">
-      <c r="A44" s="1"/>
-      <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
+      <c r="A44" s="3">
+        <v>45925.0</v>
+      </c>
+      <c r="B44" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="C44" s="19" t="s">
+        <v>89</v>
+      </c>
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>
       <c r="F44" s="2"/>
@@ -1766,9 +2209,15 @@
       <c r="Z44" s="2"/>
     </row>
     <row r="45" ht="39.75" customHeight="1">
-      <c r="A45" s="1"/>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
+      <c r="A45" s="3">
+        <v>46020.0</v>
+      </c>
+      <c r="B45" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="C45" s="19" t="s">
+        <v>91</v>
+      </c>
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
       <c r="F45" s="2"/>
@@ -1794,9 +2243,15 @@
       <c r="Z45" s="2"/>
     </row>
     <row r="46" ht="39.75" customHeight="1">
-      <c r="A46" s="1"/>
-      <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
+      <c r="A46" s="3">
+        <v>45724.0</v>
+      </c>
+      <c r="B46" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="C46" s="19" t="s">
+        <v>93</v>
+      </c>
       <c r="D46" s="2"/>
       <c r="E46" s="2"/>
       <c r="F46" s="2"/>
@@ -1822,9 +2277,15 @@
       <c r="Z46" s="2"/>
     </row>
     <row r="47" ht="39.75" customHeight="1">
-      <c r="A47" s="1"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
+      <c r="A47" s="3">
+        <v>46087.0</v>
+      </c>
+      <c r="B47" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="C47" s="19" t="s">
+        <v>95</v>
+      </c>
       <c r="D47" s="2"/>
       <c r="E47" s="2"/>
       <c r="F47" s="2"/>
@@ -1850,9 +2311,15 @@
       <c r="Z47" s="2"/>
     </row>
     <row r="48" ht="39.75" customHeight="1">
-      <c r="A48" s="1"/>
-      <c r="B48" s="2"/>
-      <c r="C48" s="2"/>
+      <c r="A48" s="3">
+        <v>46082.0</v>
+      </c>
+      <c r="B48" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="C48" s="19" t="s">
+        <v>97</v>
+      </c>
       <c r="D48" s="2"/>
       <c r="E48" s="2"/>
       <c r="F48" s="2"/>
@@ -1878,9 +2345,15 @@
       <c r="Z48" s="2"/>
     </row>
     <row r="49" ht="39.75" customHeight="1">
-      <c r="A49" s="1"/>
-      <c r="B49" s="2"/>
-      <c r="C49" s="2"/>
+      <c r="A49" s="3">
+        <v>46087.0</v>
+      </c>
+      <c r="B49" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>99</v>
+      </c>
       <c r="D49" s="2"/>
       <c r="E49" s="2"/>
       <c r="F49" s="2"/>
@@ -1906,9 +2379,15 @@
       <c r="Z49" s="2"/>
     </row>
     <row r="50" ht="39.75" customHeight="1">
-      <c r="A50" s="1"/>
-      <c r="B50" s="2"/>
-      <c r="C50" s="2"/>
+      <c r="A50" s="3">
+        <v>46083.0</v>
+      </c>
+      <c r="B50" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>101</v>
+      </c>
       <c r="D50" s="2"/>
       <c r="E50" s="2"/>
       <c r="F50" s="2"/>
@@ -1934,9 +2413,15 @@
       <c r="Z50" s="2"/>
     </row>
     <row r="51" ht="39.75" customHeight="1">
-      <c r="A51" s="1"/>
-      <c r="B51" s="2"/>
-      <c r="C51" s="2"/>
+      <c r="A51" s="3">
+        <v>46086.0</v>
+      </c>
+      <c r="B51" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>103</v>
+      </c>
       <c r="D51" s="2"/>
       <c r="E51" s="2"/>
       <c r="F51" s="2"/>
@@ -28536,21 +29021,59 @@
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="B2"/>
-    <hyperlink r:id="rId2" ref="B4"/>
-    <hyperlink r:id="rId3" ref="B5"/>
-    <hyperlink r:id="rId4" ref="B6"/>
-    <hyperlink r:id="rId5" ref="B7"/>
-    <hyperlink r:id="rId6" ref="B8"/>
-    <hyperlink r:id="rId7" ref="B9"/>
-    <hyperlink r:id="rId8" ref="B10"/>
-    <hyperlink r:id="rId9" ref="B11"/>
-    <hyperlink r:id="rId10" ref="B12"/>
-    <hyperlink r:id="rId11" ref="B13"/>
-    <hyperlink r:id="rId12" ref="B14"/>
+    <hyperlink r:id="rId2" ref="B3"/>
+    <hyperlink r:id="rId3" ref="B4"/>
+    <hyperlink r:id="rId4" ref="B5"/>
+    <hyperlink r:id="rId5" ref="B6"/>
+    <hyperlink r:id="rId6" ref="B7"/>
+    <hyperlink r:id="rId7" ref="B8"/>
+    <hyperlink r:id="rId8" ref="B9"/>
+    <hyperlink r:id="rId9" ref="B10"/>
+    <hyperlink r:id="rId10" ref="B11"/>
+    <hyperlink r:id="rId11" ref="B12"/>
+    <hyperlink r:id="rId12" ref="B13"/>
+    <hyperlink r:id="rId13" ref="B14"/>
+    <hyperlink r:id="rId14" ref="B15"/>
+    <hyperlink r:id="rId15" ref="B16"/>
+    <hyperlink r:id="rId16" ref="B17"/>
+    <hyperlink r:id="rId17" ref="B18"/>
+    <hyperlink r:id="rId18" ref="B19"/>
+    <hyperlink r:id="rId19" ref="B20"/>
+    <hyperlink r:id="rId20" ref="B21"/>
+    <hyperlink r:id="rId21" ref="B22"/>
+    <hyperlink r:id="rId22" ref="B23"/>
+    <hyperlink r:id="rId23" ref="B24"/>
+    <hyperlink r:id="rId24" ref="B25"/>
+    <hyperlink r:id="rId25" ref="B26"/>
+    <hyperlink r:id="rId26" location="IA_dans_le_jeu_video_Le_grand_craquage_de_2025" ref="B27"/>
+    <hyperlink r:id="rId27" ref="B28"/>
+    <hyperlink r:id="rId28" ref="B29"/>
+    <hyperlink r:id="rId29" ref="B30"/>
+    <hyperlink r:id="rId30" ref="B31"/>
+    <hyperlink r:id="rId31" ref="B32"/>
+    <hyperlink r:id="rId32" ref="B33"/>
+    <hyperlink r:id="rId33" ref="B34"/>
+    <hyperlink r:id="rId34" ref="B35"/>
+    <hyperlink r:id="rId35" ref="B36"/>
+    <hyperlink r:id="rId36" ref="B37"/>
+    <hyperlink r:id="rId37" ref="B38"/>
+    <hyperlink r:id="rId38" ref="B39"/>
+    <hyperlink r:id="rId39" ref="B40"/>
+    <hyperlink r:id="rId40" ref="B41"/>
+    <hyperlink r:id="rId41" ref="B42"/>
+    <hyperlink r:id="rId42" ref="B43"/>
+    <hyperlink r:id="rId43" ref="B44"/>
+    <hyperlink r:id="rId44" ref="B45"/>
+    <hyperlink r:id="rId45" ref="B46"/>
+    <hyperlink r:id="rId46" ref="B47"/>
+    <hyperlink r:id="rId47" ref="B48"/>
+    <hyperlink r:id="rId48" ref="B49"/>
+    <hyperlink r:id="rId49" ref="B50"/>
+    <hyperlink r:id="rId50" ref="B51"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <drawing r:id="rId13"/>
+  <drawing r:id="rId51"/>
 </worksheet>
 </file>
</xml_diff>